<commit_message>
Add .gitignore, PRD, and summaries; implement read_excel.py for Excel updates
</commit_message>
<xml_diff>
--- a/Suivi_Affaires_EGSA.xlsx
+++ b/Suivi_Affaires_EGSA.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +59,23 @@
       <u val="single"/>
     </font>
     <font/>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -92,8 +107,28 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF4444"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFA500"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -115,11 +150,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,6 +211,105 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -528,166 +676,208 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:W10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
-    <col width="45" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="45" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>Prochaine Action</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>Date Ouverture</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="15" t="inlineStr">
         <is>
           <t>Date Limite</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="15" t="inlineStr">
         <is>
           <t>Date Dernière MAJ</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="15" t="inlineStr">
         <is>
           <t>Historique</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="15" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="N1" s="15" t="inlineStr">
         <is>
           <t>Date Clôture</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="O1" s="15" t="inlineStr">
         <is>
           <t>Temps passé</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="P1" s="15" t="inlineStr">
         <is>
           <t>Dossier</t>
+        </is>
+      </c>
+      <c r="Q1" s="15" t="inlineStr">
+        <is>
+          <t>Date Alerte</t>
+        </is>
+      </c>
+      <c r="R1" s="15" t="inlineStr">
+        <is>
+          <t>Origine</t>
+        </is>
+      </c>
+      <c r="S1" s="15" t="inlineStr">
+        <is>
+          <t>Imprévu</t>
+        </is>
+      </c>
+      <c r="T1" s="15" t="inlineStr">
+        <is>
+          <t>Date Prochaine Action</t>
+        </is>
+      </c>
+      <c r="U1" s="15" t="inlineStr">
+        <is>
+          <t>Bloquant</t>
+        </is>
+      </c>
+      <c r="V1" s="15" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="W1" s="15" t="inlineStr">
+        <is>
+          <t>Semaine N°</t>
         </is>
       </c>
     </row>
     <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="42" t="inlineStr">
         <is>
           <t>AFF-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Courrier BIG Informatique</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="42" t="inlineStr">
         <is>
           <t>Courrier</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="42" t="inlineStr">
         <is>
           <t>Contestation de la hausse tarifaire de maintenance</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="42" t="inlineStr">
         <is>
           <t>Clôturée — Transmise à la direction</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="42" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="42" t="inlineStr">
         <is>
           <t>Aucune — Dossier transmis à la Direction des Finances</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="42" t="inlineStr">
         <is>
           <t>Yazid</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="42" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="42" t="inlineStr">
         <is>
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="42" t="inlineStr">
         <is>
           <t>2026-04-13</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="42" t="inlineStr">
         <is>
           <t>01/04 : Courrier rédigé
 10/04 : Signé par le directeur
@@ -698,289 +888,415 @@
 13/04 : Dossier transmis à la Direction des Finances — affaire hors de notre périmètre désormais</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="42" t="inlineStr">
         <is>
           <t>Le gérant de BIG Informatique a réagi par téléphone. Affaire escaladée à la Direction des Finances. Plus de notre ressort.</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="42" t="inlineStr">
         <is>
           <t>2026-04-13</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="42" t="inlineStr">
         <is>
           <t>Plusieurs jours (rédaction + validation + envoi)</t>
         </is>
       </c>
-      <c r="P2" s="13" t="inlineStr">
-        <is>
-          <t>C:\Users\hp\Desktop\YYYYYYY\Suivi_Affaires_EGSA\AFF-001_BIG_Informatique</t>
-        </is>
+      <c r="P2" s="43" t="inlineStr">
+        <is>
+          <t>C:\Users\hp\Desktop\YYYYYYY\Suivi_Affaire_EGSA\AFF-001_BIG_Informatique</t>
+        </is>
+      </c>
+      <c r="Q2" s="42" t="n"/>
+      <c r="R2" s="42" t="inlineStr">
+        <is>
+          <t>Fournisseur</t>
+        </is>
+      </c>
+      <c r="S2" s="42" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T2" s="42" t="n"/>
+      <c r="U2" s="42" t="n"/>
+      <c r="V2" s="42" t="inlineStr">
+        <is>
+          <t>BIG, Courrier, Contestation</t>
+        </is>
+      </c>
+      <c r="W2" s="42" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>AFF-002</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="44" t="inlineStr">
         <is>
           <t>Réparation Netbox Aéroport</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="44" t="inlineStr">
         <is>
           <t>Réparation</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>6 mini PC (Netbox) envoyés par un aéroport pour diagnostic et réparation</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="44" t="inlineStr">
         <is>
           <t>En attente</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="44" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="44" t="inlineStr">
         <is>
           <t>Vérifier l'avancement du diagnostic chez le technicien</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="44" t="inlineStr">
         <is>
           <t>Technicien</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="44" t="inlineStr">
         <is>
           <t>2026-04-05</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="44" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="44" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="44" t="inlineStr">
         <is>
           <t>05/04 : 6 Netbox réceptionnées
 05/04 : Remises au technicien pour diagnostic</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="44" t="inlineStr">
         <is>
           <t>Aucun retour du technicien depuis 1 semaine</t>
         </is>
       </c>
-      <c r="P3" s="14" t="n"/>
+      <c r="N3" s="44" t="n"/>
+      <c r="O3" s="44" t="n"/>
+      <c r="P3" s="44" t="n"/>
+      <c r="Q3" s="44" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="R3" s="44" t="inlineStr">
+        <is>
+          <t>Client — Aéroport</t>
+        </is>
+      </c>
+      <c r="S3" s="44" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T3" s="44" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="U3" s="44" t="inlineStr">
+        <is>
+          <t>Aucun retour du technicien depuis 9 jours</t>
+        </is>
+      </c>
+      <c r="V3" s="44" t="inlineStr">
+        <is>
+          <t>Netbox, Aéroport, Réparation</t>
+        </is>
+      </c>
+      <c r="W3" s="44" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>AFF-003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="45" t="inlineStr">
         <is>
           <t>Cahier des charges technique 2026</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="45" t="inlineStr">
         <is>
           <t>Appel d'offres</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="45" t="inlineStr">
         <is>
           <t>Conception du cahier des charges technique pour l'année 2026 incluant les lots Dev + Sécurité</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="45" t="inlineStr">
         <is>
           <t>En cours</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="45" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="45" t="inlineStr">
         <is>
           <t>Finaliser les lots après réunion et lever les questions en suspens par lot</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="45" t="inlineStr">
         <is>
           <t>Yazid</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="45" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="45" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="45" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="45" t="inlineStr">
         <is>
           <t>12/04 : Collègue a envoyé 10 lots par mail
 12/04 : Remarques faites sur les lots
 12/04 : Réunion tenue — questions en suspens identifiées par lot</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" s="45" t="inlineStr">
         <is>
           <t>Collègue a proposé 10 lots. Remarques transmises. Réunion faite.</t>
         </is>
       </c>
-      <c r="P4" s="14" t="n"/>
+      <c r="N4" s="46" t="n"/>
+      <c r="O4" s="46" t="n"/>
+      <c r="P4" s="46" t="n"/>
+      <c r="Q4" s="46" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="R4" s="46" t="inlineStr">
+        <is>
+          <t>Interne</t>
+        </is>
+      </c>
+      <c r="S4" s="46" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T4" s="46" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="U4" s="46" t="inlineStr">
+        <is>
+          <t>Questions en suspens par lot — à lever avant finalisation</t>
+        </is>
+      </c>
+      <c r="V4" s="46" t="inlineStr">
+        <is>
+          <t>CDC2026, AppelOffres</t>
+        </is>
+      </c>
+      <c r="W4" s="46" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>AFF-004</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="47" t="inlineStr">
         <is>
           <t>CDC 2026 — Lot N°1 : PCs Bureau</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="47" t="inlineStr">
         <is>
           <t>Appel d'offres / Recherche</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="47" t="inlineStr">
         <is>
           <t>Questions en suspens pour le Lot 1 (PCs bureau)</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="47" t="inlineStr">
         <is>
           <t>À traiter</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="47" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="47" t="inlineStr">
         <is>
           <t>Répondre aux questions : DVD+RW optionnel ? Port VGA encore commercialisé ?</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="47" t="inlineStr">
         <is>
           <t>Yazid</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="J5" s="47" t="inlineStr"/>
+      <c r="K5" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="47" t="inlineStr">
         <is>
           <t>12/04 : Questions identifiées après réunion</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="M5" s="47" t="inlineStr">
         <is>
           <t>❓ DVD+RW : à laisser optionnel ?
 ❓ VGA : encore commercialisé sur le marché actuel ?</t>
         </is>
       </c>
-      <c r="P5" s="14" t="n"/>
+      <c r="N5" s="47" t="n"/>
+      <c r="O5" s="47" t="n"/>
+      <c r="P5" s="47" t="n"/>
+      <c r="Q5" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="R5" s="47" t="inlineStr">
+        <is>
+          <t>Interne</t>
+        </is>
+      </c>
+      <c r="S5" s="47" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T5" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="U5" s="47" t="inlineStr">
+        <is>
+          <t>VGA encore commercialisé ? DVD+RW optionnel ? — à vérifier marché</t>
+        </is>
+      </c>
+      <c r="V5" s="47" t="inlineStr">
+        <is>
+          <t>CDC2026, Lot1, PCs</t>
+        </is>
+      </c>
+      <c r="W5" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>AFF-005</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>CDC 2026 — Lot N°2 : PCs Architectes</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>Appel d'offres / Recherche</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="47" t="inlineStr">
         <is>
           <t>Définir la configuration des PCs pour les architectes</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="47" t="inlineStr">
         <is>
           <t>À traiter</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="47" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="47" t="inlineStr">
         <is>
           <t>Répondre aux questions de configuration pour les postes architectes</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="47" t="inlineStr">
         <is>
           <t>Yazid</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="J6" s="47" t="inlineStr"/>
+      <c r="K6" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L6" s="47" t="inlineStr">
         <is>
           <t>12/04 : Questions identifiées après réunion</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="M6" s="47" t="inlineStr">
         <is>
           <t>❓ Combien de PCs ?
 ❓ Comment ils travaillent actuellement ?
@@ -988,216 +1304,443 @@
 ❓ AutoCAD seulement ou autres logiciels ?</t>
         </is>
       </c>
-      <c r="P6" s="14" t="n"/>
+      <c r="N6" s="47" t="n"/>
+      <c r="O6" s="47" t="n"/>
+      <c r="P6" s="47" t="n"/>
+      <c r="Q6" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="R6" s="47" t="inlineStr">
+        <is>
+          <t>Interne</t>
+        </is>
+      </c>
+      <c r="S6" s="47" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T6" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="U6" s="47" t="inlineStr">
+        <is>
+          <t>Nombre de PCs ? Logiciels utilisés ? Usage 2D/3D ? — à définir</t>
+        </is>
+      </c>
+      <c r="V6" s="47" t="inlineStr">
+        <is>
+          <t>CDC2026, Lot2, Architectes</t>
+        </is>
+      </c>
+      <c r="W6" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>AFF-006</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="47" t="inlineStr">
         <is>
           <t>CDC 2026 — Lot N°2 : Laptops Développeurs</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="47" t="inlineStr">
         <is>
           <t>Appel d'offres / Recherche</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="47" t="inlineStr">
         <is>
           <t>Définir la configuration des laptops pour les développeurs</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="47" t="inlineStr">
         <is>
           <t>À traiter</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="47" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="47" t="inlineStr">
         <is>
           <t>Répondre aux questions de configuration pour les laptops dev</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="47" t="inlineStr">
         <is>
           <t>Yazid</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="J7" s="47" t="inlineStr"/>
+      <c r="K7" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="L7" s="47" t="inlineStr">
         <is>
           <t>12/04 : Questions identifiées après réunion</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="M7" s="47" t="inlineStr">
         <is>
           <t>❓ Laptop avec ou sans station d'accueil bureau ?
 ❓ Quelle configuration technique recommandée ?</t>
         </is>
       </c>
-      <c r="P7" s="14" t="n"/>
+      <c r="N7" s="47" t="n"/>
+      <c r="O7" s="47" t="n"/>
+      <c r="P7" s="47" t="n"/>
+      <c r="Q7" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="R7" s="47" t="inlineStr">
+        <is>
+          <t>Interne</t>
+        </is>
+      </c>
+      <c r="S7" s="47" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T7" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="U7" s="47" t="inlineStr">
+        <is>
+          <t>Avec ou sans station d'accueil ? Config technique — à définir</t>
+        </is>
+      </c>
+      <c r="V7" s="47" t="inlineStr">
+        <is>
+          <t>CDC2026, Lot2, Laptops, Dev</t>
+        </is>
+      </c>
+      <c r="W7" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>AFF-007</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>CDC 2026 — Lots N°3 &amp; 4 : Stockage SSD</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Appel d'offres / Décision</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Décider si on impose un minimum de 256 Go SSD ou si on le retire pour élargir les candidatures</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>À décider</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="47" t="inlineStr">
         <is>
           <t>Trancher : garder '256 Go SSD minimum' ou retirer la contrainte pour maximiser les offres</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="47" t="inlineStr">
         <is>
           <t>Yazid</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="I8" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr"/>
-      <c r="K8" s="8" t="inlineStr">
+      <c r="J8" s="47" t="inlineStr"/>
+      <c r="K8" s="47" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="L8" s="8" t="inlineStr">
+      <c r="L8" s="47" t="inlineStr">
         <is>
           <t>12/04 : Question soulevée après réunion</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="M8" s="47" t="inlineStr">
         <is>
           <t>⚖️ Garder '256 Go SSD min' = qualité garantie mais risque de réduire concurrence
 Retirer le min = plus d'offres potentielles mais qualité variable</t>
         </is>
       </c>
-      <c r="P8" s="14" t="n"/>
+      <c r="N8" s="47" t="n"/>
+      <c r="O8" s="47" t="n"/>
+      <c r="P8" s="47" t="n"/>
+      <c r="Q8" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="R8" s="47" t="inlineStr">
+        <is>
+          <t>Interne</t>
+        </is>
+      </c>
+      <c r="S8" s="47" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T8" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="U8" s="47" t="inlineStr">
+        <is>
+          <t>Décision 256 Go SSD minimum : garder ou retirer ?</t>
+        </is>
+      </c>
+      <c r="V8" s="47" t="inlineStr">
+        <is>
+          <t>CDC2026, Lot3, Lot4, SSD</t>
+        </is>
+      </c>
+      <c r="W8" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="42" t="inlineStr">
         <is>
           <t>AFF-008</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="42" t="inlineStr">
         <is>
           <t>Préparation salle de formation — Regroupement comptables</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>À la volée</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>Câblage et préparation de la salle de formation pour le regroupement des comptables de tous les aéroports prévu dans la semaine</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="42" t="inlineStr">
         <is>
           <t>Clôturée</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="42" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="42" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="42" t="inlineStr">
         <is>
           <t>Yazid</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="I9" s="42" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="J9" s="42" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="L9" s="11" t="inlineStr">
+      <c r="K9" s="42" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="L9" s="42" t="inlineStr">
         <is>
           <t>12/04 : Appel reçu à 08h00 — câblage et préparation salle de formation effectués toute la matinée
-13/04 : Installation finalisée pour le 2ème jour du regroupement (comptables + commerciaux)</t>
-        </is>
-      </c>
-      <c r="M9" s="11" t="inlineStr">
+13/04 : Installation finalisée pour le 2ème jour du regroupement (comptables + commerciaux)
+14/04 : Assistance à la réunion commerciale dans la salle de formation</t>
+        </is>
+      </c>
+      <c r="M9" s="42" t="inlineStr">
         <is>
           <t>Tâche à la volée — non planifiée</t>
         </is>
       </c>
-      <c r="N9" s="11" t="inlineStr">
+      <c r="N9" s="42" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="O9" s="11" t="inlineStr">
-        <is>
-          <t>Matinée 12/04 (~4h) + installation 13/04</t>
-        </is>
-      </c>
-      <c r="P9" s="14" t="n"/>
+      <c r="O9" s="42" t="inlineStr">
+        <is>
+          <t>Matinée 12/04 (~4h) + installation 13/04 + assistance réunion 14/04</t>
+        </is>
+      </c>
+      <c r="P9" s="42" t="n"/>
+      <c r="Q9" s="42" t="n"/>
+      <c r="R9" s="42" t="inlineStr">
+        <is>
+          <t>Direction — Imprévu</t>
+        </is>
+      </c>
+      <c r="S9" s="42" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="T9" s="42" t="n"/>
+      <c r="U9" s="42" t="n"/>
+      <c r="V9" s="42" t="inlineStr">
+        <is>
+          <t>Formation, Regroupement, Salle</t>
+        </is>
+      </c>
+      <c r="W9" s="42" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="47" t="inlineStr">
+        <is>
+          <t>AFF-009</t>
+        </is>
+      </c>
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t>Analyse base de données ERP</t>
+        </is>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr">
+        <is>
+          <t>Analyse de la base de données (.bak) fournie par la collègue pour le futur ERP</t>
+        </is>
+      </c>
+      <c r="E10" s="47" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="F10" s="47" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G10" s="47" t="inlineStr">
+        <is>
+          <t>Restaurer le .bak et analyser la structure + contenu de la base</t>
+        </is>
+      </c>
+      <c r="H10" s="47" t="inlineStr">
+        <is>
+          <t>Yazid</t>
+        </is>
+      </c>
+      <c r="I10" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="J10" s="47" t="n"/>
+      <c r="K10" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="L10" s="47" t="inlineStr">
+        <is>
+          <t>14/04 : Base de données reçue de la collègue — analyse à démarrer en urgence
+14/04 : Base de données .bak reçue de la collègue — analyse à démarrer en urgence</t>
+        </is>
+      </c>
+      <c r="M10" s="47" t="inlineStr">
+        <is>
+          <t>Fichier au format .bak (backup SQL Server)</t>
+        </is>
+      </c>
+      <c r="N10" s="47" t="n"/>
+      <c r="O10" s="47" t="n"/>
+      <c r="P10" s="47" t="n"/>
+      <c r="Q10" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="R10" s="47" t="inlineStr">
+        <is>
+          <t>Collègue</t>
+        </is>
+      </c>
+      <c r="S10" s="47" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="T10" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U10" s="47" t="inlineStr">
+        <is>
+          <t>Fichier .bak reçu — besoin restauration SQL Server pour analyse</t>
+        </is>
+      </c>
+      <c r="V10" s="47" t="inlineStr">
+        <is>
+          <t>ERP, BDD, Analyse</t>
+        </is>
+      </c>
+      <c r="W10" s="47" t="n">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Add script for generating EGSA affairs report and create initial report file  - Implemented `print_suivi2.py` to read and format data from an Excel sheet. - Added functionality to display affairs with details such as ID, Title, Status, Priority, and deadlines. - Included urgency flags based on deadline proximity. - Created `rapport.txt` to store the generated report output.
</commit_message>
<xml_diff>
--- a/Suivi_Affaires_EGSA.xlsx
+++ b/Suivi_Affaires_EGSA.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="12">
     <font>
       <name val="Calibri"/>
@@ -168,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -311,6 +313,16 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -676,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W10"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -844,7 +856,7 @@
       </c>
       <c r="E2" s="42" t="inlineStr">
         <is>
-          <t>Clôturée — Transmise à la direction</t>
+          <t>Clôturée — Courrier traité, réponse BIG Informatique attendue</t>
         </is>
       </c>
       <c r="F2" s="42" t="inlineStr">
@@ -854,7 +866,7 @@
       </c>
       <c r="G2" s="42" t="inlineStr">
         <is>
-          <t>Aucune — Dossier transmis à la Direction des Finances</t>
+          <t>Attendre réponse formelle de BIG Informatique — Démarrer en parallèle le projet ERP (AFF-009)</t>
         </is>
       </c>
       <c r="H2" s="42" t="inlineStr">
@@ -872,10 +884,8 @@
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="K2" s="42" t="inlineStr">
-        <is>
-          <t>2026-04-13</t>
-        </is>
+      <c r="K2" s="48" t="n">
+        <v>46127</v>
       </c>
       <c r="L2" s="42" t="inlineStr">
         <is>
@@ -885,12 +895,16 @@
 13/04 : Mail envoyé au gérant avec courrier officiel de contestation + proforma en PJ
 13/04 : Mail envoyé avec courrier officiel + proforma en PJ
 13/04 : Gérant BIG a appelé — juge le mail disproportionné
-13/04 : Dossier transmis à la Direction des Finances — affaire hors de notre périmètre désormais</t>
+13/04 : Dossier transmis à la Direction des Finances — affaire hors de notre périmètre désormais
+15/04/2026 — Suite à réception du courrier officiel, le DG de BIG Informatique a appelé et exprimé son mécontentement. Risque élevé de non-renouvellement du contrat de maintenance 2026/2027. Décision prise : démarrer le projet ERP en alternative à la dépendance BIG Informatique.
+15/04/2026 — Suite à réception du courrier officiel, le DG de BIG Informatique a appelé et exprimé son mécontentement. Risque élevé de non-renouvellement du contrat de maintenance 2026/2027. Décision prise : démarrer le projet ERP en alternative à la dépendance BIG Informatique.</t>
         </is>
       </c>
       <c r="M2" s="42" t="inlineStr">
         <is>
-          <t>Le gérant de BIG Informatique a réagi par téléphone. Affaire escaladée à la Direction des Finances. Plus de notre ressort.</t>
+          <t>Le gérant de BIG Informatique a réagi par téléphone. Affaire escaladée à la Direction des Finances. Plus de notre ressort.
+15/04/2026 — DG BIG mécontent après réception courrier. Contrat maintenance 2026/2027 compromis. Transition vers projet ERP envisagée.
+15/04/2026 — DG BIG mécontent après réception courrier. Contrat maintenance 2026/2027 compromis. Transition vers projet ERP envisagée.</t>
         </is>
       </c>
       <c r="N2" s="42" t="inlineStr">
@@ -908,7 +922,9 @@
           <t>C:\Users\hp\Desktop\YYYYYYY\Suivi_Affaire_EGSA\AFF-001_BIG_Informatique</t>
         </is>
       </c>
-      <c r="Q2" s="42" t="n"/>
+      <c r="Q2" s="48" t="n">
+        <v>46135</v>
+      </c>
       <c r="R2" s="42" t="inlineStr">
         <is>
           <t>Fournisseur</t>
@@ -919,11 +935,17 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T2" s="42" t="n"/>
-      <c r="U2" s="42" t="n"/>
+      <c r="T2" s="48" t="n">
+        <v>46135</v>
+      </c>
+      <c r="U2" s="42" t="inlineStr">
+        <is>
+          <t>Réponse formelle de BIG Informatique en attente — risque de rupture contractuelle</t>
+        </is>
+      </c>
       <c r="V2" s="42" t="inlineStr">
         <is>
-          <t>BIG, Courrier, Contestation</t>
+          <t>BIG, Courrier, Contestation, ERP</t>
         </is>
       </c>
       <c r="W2" s="42" t="n">
@@ -963,7 +985,7 @@
       </c>
       <c r="G3" s="44" t="inlineStr">
         <is>
-          <t>Vérifier l'avancement du diagnostic chez le technicien</t>
+          <t>Dimanche 19/04 : vérifier l'avancement du diagnostic Netbox avec le technicien</t>
         </is>
       </c>
       <c r="H3" s="44" t="inlineStr">
@@ -976,20 +998,18 @@
           <t>2026-04-05</t>
         </is>
       </c>
-      <c r="J3" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-12</t>
-        </is>
-      </c>
-      <c r="K3" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-12</t>
-        </is>
+      <c r="J3" s="49" t="n">
+        <v>46131</v>
+      </c>
+      <c r="K3" s="49" t="n">
+        <v>46127</v>
       </c>
       <c r="L3" s="44" t="inlineStr">
         <is>
           <t>05/04 : 6 Netbox réceptionnées
-05/04 : Remises au technicien pour diagnostic</t>
+05/04 : Remises au technicien pour diagnostic
+15/04/2026 — Délai prolongé : techniciens mobilisés pour le regroupement des comptables et commerciaux toute la semaine du 07/04 au 10/04. Nouvelle date cible : dimanche 19/04/2026.
+15/04/2026 — Délai prolongé : techniciens mobilisés pour le regroupement des comptables et commerciaux toute la semaine du 07/04 au 10/04. Nouvelle date cible : dimanche 19/04/2026.</t>
         </is>
       </c>
       <c r="M3" s="44" t="inlineStr">
@@ -1000,10 +1020,8 @@
       <c r="N3" s="44" t="n"/>
       <c r="O3" s="44" t="n"/>
       <c r="P3" s="44" t="n"/>
-      <c r="Q3" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
+      <c r="Q3" s="49" t="n">
+        <v>46131</v>
       </c>
       <c r="R3" s="44" t="inlineStr">
         <is>
@@ -1015,14 +1033,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T3" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
+      <c r="T3" s="49" t="n">
+        <v>46131</v>
       </c>
       <c r="U3" s="44" t="inlineStr">
         <is>
-          <t>Aucun retour du technicien depuis 9 jours</t>
+          <t>Techniciens occupés avec regroupement comptables/commerciaux — Délai prolongé au 19/04/2026</t>
         </is>
       </c>
       <c r="V3" s="44" t="inlineStr">
@@ -1675,7 +1691,7 @@
       </c>
       <c r="G10" s="47" t="inlineStr">
         <is>
-          <t>Restaurer le .bak et analyser la structure + contenu de la base</t>
+          <t>1) Appeler le collègue pour identifier la base de données de production 2) Restaurer le .bak sur SQL Server et démarrer l'analyse de structure</t>
         </is>
       </c>
       <c r="H10" s="47" t="inlineStr">
@@ -1689,15 +1705,15 @@
         </is>
       </c>
       <c r="J10" s="47" t="n"/>
-      <c r="K10" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
+      <c r="K10" s="50" t="n">
+        <v>46127</v>
       </c>
       <c r="L10" s="47" t="inlineStr">
         <is>
           <t>14/04 : Base de données reçue de la collègue — analyse à démarrer en urgence
-14/04 : Base de données .bak reçue de la collègue — analyse à démarrer en urgence</t>
+14/04 : Base de données .bak reçue de la collègue — analyse à démarrer en urgence
+15/04/2026 — Problème identifié : deux bases de données présentes. Incertitude sur laquelle est utilisée en production. À clarifier avec le collègue avant toute analyse ou restauration.
+15/04/2026 — Problème identifié : deux bases de données présentes. Incertitude sur laquelle est utilisée en production. À clarifier avec le collègue avant toute analyse ou restauration.</t>
         </is>
       </c>
       <c r="M10" s="47" t="inlineStr">
@@ -1708,10 +1724,8 @@
       <c r="N10" s="47" t="n"/>
       <c r="O10" s="47" t="n"/>
       <c r="P10" s="47" t="n"/>
-      <c r="Q10" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
+      <c r="Q10" s="50" t="n">
+        <v>46127</v>
       </c>
       <c r="R10" s="47" t="inlineStr">
         <is>
@@ -1723,14 +1737,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T10" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
+      <c r="T10" s="50" t="n">
+        <v>46127</v>
       </c>
       <c r="U10" s="47" t="inlineStr">
         <is>
-          <t>Fichier .bak reçu — besoin restauration SQL Server pour analyse</t>
+          <t>Deux bases de données disponibles — impossible de savoir laquelle est en production sans appel collègue</t>
         </is>
       </c>
       <c r="V10" s="47" t="inlineStr">
@@ -1739,6 +1751,268 @@
         </is>
       </c>
       <c r="W10" s="47" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AFF-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tests des PC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>À la volée</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Tester les PC disponibles — validation du matériel avant déploiement.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Clôturée</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Yazid</t>
+        </is>
+      </c>
+      <c r="I11" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="J11" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="K11" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>15/04/2026 — Tâche ajoutée : tests PC à réaliser aujourd'hui.
+15/04/2026 — Tests terminés. Tous les PCs sont fonctionnels.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Tous les PCs testés et validés le 15/04/2026. 8 mini PCs à distribuer aux comptables présents : Comptable 1 = 2 PCs, Comptable 2 = 4 PCs, Comptable 3 = 2 PCs. → Décharges à préparer et signer AVANT remise du matériel (voir AFF-012).</t>
+        </is>
+      </c>
+      <c r="N11" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="Q11" s="51" t="n"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Imprévu</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="T11" s="51" t="n"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Tests, Matériel</t>
+        </is>
+      </c>
+      <c r="W11" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AFF-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Entretien avec le commercial</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>À la volée</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Appel ou rencontre avec le commercial — matin ou après-midi du 15/04/2026.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>À traiter</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Appeler ou rencontrer le commercial aujourd'hui (matin ou après-midi)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Yazid</t>
+        </is>
+      </c>
+      <c r="I12" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="J12" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="K12" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>15/04/2026 — Tâche ajoutée : entretien commercial à planifier aujourd'hui.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Prévoir matin ou après-midi selon disponibilité.</t>
+        </is>
+      </c>
+      <c r="Q12" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Imprévu</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="T12" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Commercial, Réunion</t>
+        </is>
+      </c>
+      <c r="W12" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AFF-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Décharges remise mini PCs aux comptables</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>À la volée</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Préparer les 3 décharges de remise de matériel pour les comptables du regroupement. Distribution : Comptable 1 = 2 mini PCs, Comptable 2 = 4 mini PCs, Comptable 3 = 2 mini PCs. Total = 8 mini PCs. Les décharges doivent être signées AVANT que les comptables repartent.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>À traiter</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1) Préparer les 3 décharges (nom, quantité, modèle, n° série si disponible) 2) Les faire signer par les 3 comptables avant leur départ</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Yazid</t>
+        </is>
+      </c>
+      <c r="I13" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="J13" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="K13" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>15/04/2026 — Tests PC terminés. 8 mini PCs à distribuer : 2 + 4 + 2. Décharges obligatoires avant remise.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Comptable 1 : 2 | Comptable 2 : 4 | Comptable 3 : 2 — Total : 8 mini PCs</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Imprévu</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="T13" s="51" t="n">
+        <v>46127</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Décharges non encore préparées — bloquer la remise du matériel jusqu'à signature</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Matériel, Décharge, Comptables, Mini PC</t>
+        </is>
+      </c>
+      <c r="W13" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add multiple scripts for managing EGSA affairs, including task updates, briefings, and searches
</commit_message>
<xml_diff>
--- a/Suivi_Affaires_EGSA.xlsx
+++ b/Suivi_Affaires_EGSA.xlsx
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -323,6 +323,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -688,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1002,14 +1008,16 @@
         <v>46131</v>
       </c>
       <c r="K3" s="49" t="n">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="L3" s="44" t="inlineStr">
         <is>
           <t>05/04 : 6 Netbox réceptionnées
 05/04 : Remises au technicien pour diagnostic
 15/04/2026 — Délai prolongé : techniciens mobilisés pour le regroupement des comptables et commerciaux toute la semaine du 07/04 au 10/04. Nouvelle date cible : dimanche 19/04/2026.
-15/04/2026 — Délai prolongé : techniciens mobilisés pour le regroupement des comptables et commerciaux toute la semaine du 07/04 au 10/04. Nouvelle date cible : dimanche 19/04/2026.</t>
+15/04/2026 — Délai prolongé : techniciens mobilisés pour le regroupement des comptables et commerciaux toute la semaine du 07/04 au 10/04. Nouvelle date cible : dimanche 19/04/2026.
+20/04/2026 — Délai prolongé au jeudi 23/04/2026 (techniciens occupés)
+20/04/2026 — Reporté à fin de semaine (25/04) : techniciens toujours occupés.</t>
         </is>
       </c>
       <c r="M3" s="44" t="inlineStr">
@@ -1021,7 +1029,7 @@
       <c r="O3" s="44" t="n"/>
       <c r="P3" s="44" t="n"/>
       <c r="Q3" s="49" t="n">
-        <v>46131</v>
+        <v>46137</v>
       </c>
       <c r="R3" s="44" t="inlineStr">
         <is>
@@ -1034,11 +1042,11 @@
         </is>
       </c>
       <c r="T3" s="49" t="n">
-        <v>46131</v>
+        <v>46137</v>
       </c>
       <c r="U3" s="44" t="inlineStr">
         <is>
-          <t>Techniciens occupés avec regroupement comptables/commerciaux — Délai prolongé au 19/04/2026</t>
+          <t>Techniciens occupés — traitement prévu fin de semaine (25/04)</t>
         </is>
       </c>
       <c r="V3" s="44" t="inlineStr">
@@ -1083,7 +1091,7 @@
       </c>
       <c r="G4" s="45" t="inlineStr">
         <is>
-          <t>Finaliser les lots après réunion et lever les questions en suspens par lot</t>
+          <t>RAPPEL demain après-midi 21/04 — Finaliser les lots CDC 2026 (AFF-004, 005, 006, 007 liées)</t>
         </is>
       </c>
       <c r="H4" s="45" t="inlineStr">
@@ -1101,16 +1109,15 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="K4" s="45" t="inlineStr">
-        <is>
-          <t>2026-04-12</t>
-        </is>
+      <c r="K4" s="52" t="n">
+        <v>46132</v>
       </c>
       <c r="L4" s="45" t="inlineStr">
         <is>
           <t>12/04 : Collègue a envoyé 10 lots par mail
 12/04 : Remarques faites sur les lots
-12/04 : Réunion tenue — questions en suspens identifiées par lot</t>
+12/04 : Réunion tenue — questions en suspens identifiées par lot
+20/04/2026 — Planifié pour demain après-midi 21/04/2026. Les lots AFF-004/005/006/007 seront traités en même temps.</t>
         </is>
       </c>
       <c r="M4" s="45" t="inlineStr">
@@ -1121,10 +1128,8 @@
       <c r="N4" s="46" t="n"/>
       <c r="O4" s="46" t="n"/>
       <c r="P4" s="46" t="n"/>
-      <c r="Q4" s="46" t="inlineStr">
-        <is>
-          <t>2026-04-21</t>
-        </is>
+      <c r="Q4" s="53" t="n">
+        <v>46133</v>
       </c>
       <c r="R4" s="46" t="inlineStr">
         <is>
@@ -1136,10 +1141,8 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T4" s="46" t="inlineStr">
-        <is>
-          <t>2026-04-21</t>
-        </is>
+      <c r="T4" s="53" t="n">
+        <v>46133</v>
       </c>
       <c r="U4" s="46" t="inlineStr">
         <is>
@@ -1188,7 +1191,7 @@
       </c>
       <c r="G5" s="47" t="inlineStr">
         <is>
-          <t>Répondre aux questions : DVD+RW optionnel ? Port VGA encore commercialisé ?</t>
+          <t>Traiter avec AFF-003 — demain après-midi 21/04/2026</t>
         </is>
       </c>
       <c r="H5" s="47" t="inlineStr">
@@ -1202,14 +1205,13 @@
         </is>
       </c>
       <c r="J5" s="47" t="inlineStr"/>
-      <c r="K5" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-12</t>
-        </is>
+      <c r="K5" s="50" t="n">
+        <v>46132</v>
       </c>
       <c r="L5" s="47" t="inlineStr">
         <is>
-          <t>12/04 : Questions identifiées après réunion</t>
+          <t>12/04 : Questions identifiées après réunion
+20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.</t>
         </is>
       </c>
       <c r="M5" s="47" t="inlineStr">
@@ -1221,10 +1223,8 @@
       <c r="N5" s="47" t="n"/>
       <c r="O5" s="47" t="n"/>
       <c r="P5" s="47" t="n"/>
-      <c r="Q5" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="Q5" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="R5" s="47" t="inlineStr">
         <is>
@@ -1236,10 +1236,8 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T5" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="T5" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="U5" s="47" t="inlineStr">
         <is>
@@ -1248,7 +1246,7 @@
       </c>
       <c r="V5" s="47" t="inlineStr">
         <is>
-          <t>CDC2026, Lot1, PCs</t>
+          <t>CDC2026, Lot1, PCs, LiéeAFF-003</t>
         </is>
       </c>
       <c r="W5" s="47" t="n">
@@ -1288,7 +1286,7 @@
       </c>
       <c r="G6" s="47" t="inlineStr">
         <is>
-          <t>Répondre aux questions de configuration pour les postes architectes</t>
+          <t>Traiter avec AFF-003 — demain après-midi 21/04/2026</t>
         </is>
       </c>
       <c r="H6" s="47" t="inlineStr">
@@ -1302,14 +1300,13 @@
         </is>
       </c>
       <c r="J6" s="47" t="inlineStr"/>
-      <c r="K6" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-12</t>
-        </is>
+      <c r="K6" s="50" t="n">
+        <v>46132</v>
       </c>
       <c r="L6" s="47" t="inlineStr">
         <is>
-          <t>12/04 : Questions identifiées après réunion</t>
+          <t>12/04 : Questions identifiées après réunion
+20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.</t>
         </is>
       </c>
       <c r="M6" s="47" t="inlineStr">
@@ -1323,10 +1320,8 @@
       <c r="N6" s="47" t="n"/>
       <c r="O6" s="47" t="n"/>
       <c r="P6" s="47" t="n"/>
-      <c r="Q6" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="Q6" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="R6" s="47" t="inlineStr">
         <is>
@@ -1338,10 +1333,8 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T6" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="T6" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="U6" s="47" t="inlineStr">
         <is>
@@ -1350,7 +1343,7 @@
       </c>
       <c r="V6" s="47" t="inlineStr">
         <is>
-          <t>CDC2026, Lot2, Architectes</t>
+          <t>CDC2026, Lot2, Architectes, LiéeAFF-003</t>
         </is>
       </c>
       <c r="W6" s="47" t="n">
@@ -1390,7 +1383,7 @@
       </c>
       <c r="G7" s="47" t="inlineStr">
         <is>
-          <t>Répondre aux questions de configuration pour les laptops dev</t>
+          <t>Traiter avec AFF-003 — demain après-midi 21/04/2026</t>
         </is>
       </c>
       <c r="H7" s="47" t="inlineStr">
@@ -1404,14 +1397,13 @@
         </is>
       </c>
       <c r="J7" s="47" t="inlineStr"/>
-      <c r="K7" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-12</t>
-        </is>
+      <c r="K7" s="50" t="n">
+        <v>46132</v>
       </c>
       <c r="L7" s="47" t="inlineStr">
         <is>
-          <t>12/04 : Questions identifiées après réunion</t>
+          <t>12/04 : Questions identifiées après réunion
+20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.</t>
         </is>
       </c>
       <c r="M7" s="47" t="inlineStr">
@@ -1423,10 +1415,8 @@
       <c r="N7" s="47" t="n"/>
       <c r="O7" s="47" t="n"/>
       <c r="P7" s="47" t="n"/>
-      <c r="Q7" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="Q7" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="R7" s="47" t="inlineStr">
         <is>
@@ -1438,10 +1428,8 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T7" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="T7" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="U7" s="47" t="inlineStr">
         <is>
@@ -1450,7 +1438,7 @@
       </c>
       <c r="V7" s="47" t="inlineStr">
         <is>
-          <t>CDC2026, Lot2, Laptops, Dev</t>
+          <t>CDC2026, Lot2, Laptops, Dev, LiéeAFF-003</t>
         </is>
       </c>
       <c r="W7" s="47" t="n">
@@ -1490,7 +1478,7 @@
       </c>
       <c r="G8" s="47" t="inlineStr">
         <is>
-          <t>Trancher : garder '256 Go SSD minimum' ou retirer la contrainte pour maximiser les offres</t>
+          <t>Traiter avec AFF-003 — demain après-midi 21/04/2026</t>
         </is>
       </c>
       <c r="H8" s="47" t="inlineStr">
@@ -1504,14 +1492,13 @@
         </is>
       </c>
       <c r="J8" s="47" t="inlineStr"/>
-      <c r="K8" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-12</t>
-        </is>
+      <c r="K8" s="50" t="n">
+        <v>46132</v>
       </c>
       <c r="L8" s="47" t="inlineStr">
         <is>
-          <t>12/04 : Question soulevée après réunion</t>
+          <t>12/04 : Question soulevée après réunion
+20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.</t>
         </is>
       </c>
       <c r="M8" s="47" t="inlineStr">
@@ -1523,10 +1510,8 @@
       <c r="N8" s="47" t="n"/>
       <c r="O8" s="47" t="n"/>
       <c r="P8" s="47" t="n"/>
-      <c r="Q8" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="Q8" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="R8" s="47" t="inlineStr">
         <is>
@@ -1538,10 +1523,8 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="T8" s="47" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
+      <c r="T8" s="50" t="n">
+        <v>46133</v>
       </c>
       <c r="U8" s="47" t="inlineStr">
         <is>
@@ -1550,7 +1533,7 @@
       </c>
       <c r="V8" s="47" t="inlineStr">
         <is>
-          <t>CDC2026, Lot3, Lot4, SSD</t>
+          <t>CDC2026, Lot3, Lot4, SSD, LiéeAFF-003</t>
         </is>
       </c>
       <c r="W8" s="47" t="n">
@@ -1691,7 +1674,7 @@
       </c>
       <c r="G10" s="47" t="inlineStr">
         <is>
-          <t>1) Appeler le collègue pour identifier la base de données de production 2) Restaurer le .bak sur SQL Server et démarrer l'analyse de structure</t>
+          <t>RAPPEL demain matin 21/04 — Analyser BD ERP avec collègues + préparer résumé commercial réunion 14/04</t>
         </is>
       </c>
       <c r="H10" s="47" t="inlineStr">
@@ -1706,14 +1689,19 @@
       </c>
       <c r="J10" s="47" t="n"/>
       <c r="K10" s="50" t="n">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="L10" s="47" t="inlineStr">
         <is>
           <t>14/04 : Base de données reçue de la collègue — analyse à démarrer en urgence
 14/04 : Base de données .bak reçue de la collègue — analyse à démarrer en urgence
 15/04/2026 — Problème identifié : deux bases de données présentes. Incertitude sur laquelle est utilisée en production. À clarifier avec le collègue avant toute analyse ou restauration.
-15/04/2026 — Problème identifié : deux bases de données présentes. Incertitude sur laquelle est utilisée en production. À clarifier avec le collègue avant toute analyse ou restauration.</t>
+15/04/2026 — Problème identifié : deux bases de données présentes. Incertitude sur laquelle est utilisée en production. À clarifier avec le collègue avant toute analyse ou restauration.
+19/04/2026 — Jour sans bureau (dimanche), aucune action possibility
+20/04/2026 — A COMMENCER : appeler collègue pour identifier BD production
+20/04/2026 — Base de données restaurée en local (.bak OK). BD identifiée : base des commerciaux en production. Prochaine étape : analyse structure + résumé commercial (en groupe avec collègues).
+20/04/2026 — Planifié pour demain matin 21/04/2026 : analyse BD structure + résumé commercial réunion commerciale du 14/04.
+20/04/2026 — Planifié pour demain matin 21/04/2026 : analyse structure BD + résumé commercial réunion du 14/04.</t>
         </is>
       </c>
       <c r="M10" s="47" t="inlineStr">
@@ -1725,7 +1713,7 @@
       <c r="O10" s="47" t="n"/>
       <c r="P10" s="47" t="n"/>
       <c r="Q10" s="50" t="n">
-        <v>46127</v>
+        <v>46133</v>
       </c>
       <c r="R10" s="47" t="inlineStr">
         <is>
@@ -1738,13 +1726,9 @@
         </is>
       </c>
       <c r="T10" s="50" t="n">
-        <v>46127</v>
-      </c>
-      <c r="U10" s="47" t="inlineStr">
-        <is>
-          <t>Deux bases de données disponibles — impossible de savoir laquelle est en production sans appel collègue</t>
-        </is>
-      </c>
+        <v>46133</v>
+      </c>
+      <c r="U10" s="47" t="n"/>
       <c r="V10" s="47" t="inlineStr">
         <is>
           <t>ERP, BDD, Analyse</t>
@@ -1862,7 +1846,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1872,7 +1856,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Appeler ou rencontrer le commercial aujourd'hui (matin ou après-midi)</t>
+          <t>Rédiger résumé métier commercial (réunion 15/04) + intégrer à la conception ERP — en coordination avec AFF-009</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1887,11 +1871,13 @@
         <v>46127</v>
       </c>
       <c r="K12" s="51" t="n">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>15/04/2026 — Tâche ajoutée : entretien commercial à planifier aujourd'hui.</t>
+          <t>15/04/2026 — Tâche ajoutée : entretien commercial à planifier aujourd'hui.
+20/04/2026 — Réunion avec commercial effectuée
+20/04/2026 — Réunion du 15/04 avec le commercial confirmée. Prochaine étape : rédiger résumé métier + l'intégrer à la conception ERP (lié AFF-009). Objectif : conception ERP complète et rigoureuse.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1915,9 +1901,14 @@
       <c r="T12" s="51" t="n">
         <v>46127</v>
       </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Nécessite coordination avec AFF-009 — conception ERP à faire ensemble</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Commercial, Réunion</t>
+          <t>Commercial, Réunion, ERP, ConceptionERP, LiéeAFF-009</t>
         </is>
       </c>
       <c r="W12" t="n">
@@ -1947,7 +1938,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>À traiter</t>
+          <t>Clôturée</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1957,7 +1948,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1) Préparer les 3 décharges (nom, quantité, modèle, n° série si disponible) 2) Les faire signer par les 3 comptables avant leur départ</t>
+          <t>Affaire clôturée — Décharges signées par 3 comptables, 8 mini PC envoyés (3 aéroports)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1972,11 +1963,12 @@
         <v>46127</v>
       </c>
       <c r="K13" s="51" t="n">
-        <v>46127</v>
+        <v>46132</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>15/04/2026 — Tests PC terminés. 8 mini PCs à distribuer : 2 + 4 + 2. Décharges obligatoires avant remise.</t>
+          <t>15/04/2026 — Tests PC terminés. 8 mini PCs à distribuer : 2 + 4 + 2. Décharges obligatoires avant remise.
+20/04/2026 — CLÔTURÉ : Décharges signées, 8 mini PC envoyés dans 3 aéroports</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1984,8 +1976,9 @@
           <t>Comptable 1 : 2 | Comptable 2 : 4 | Comptable 3 : 2 — Total : 8 mini PCs</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="N13" s="51" t="n">
+        <v>46132</v>
+      </c>
       <c r="Q13" s="51" t="n">
         <v>46127</v>
       </c>
@@ -2014,6 +2007,77 @@
       </c>
       <c r="W13" t="n">
         <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AFF-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bilans mensuels — Janvier, Février, Mars</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>La directrice doit envoyer les trois bilans mensuels (J/F/M) — État des lieux</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>À traiter</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>RAPPEL demain 21/04 — Relancer la directrice pour envoi des bilans mensuels J/F/M</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Directrice</t>
+        </is>
+      </c>
+      <c r="I14" s="51" t="n">
+        <v>46132</v>
+      </c>
+      <c r="K14" s="51" t="n">
+        <v>46132</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>20/04/2026 — CRÉÉ : Affaire de suivi pour les trois bilans mensuels
+Rappel quotidien jusqu'à complération
+20/04/2026 — Rappel programmé pour demain 21/04/2026.</t>
+        </is>
+      </c>
+      <c r="Q14" s="51" t="n">
+        <v>46133</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Imprévu</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="T14" s="51" t="n">
+        <v>46133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add scripts for task management and updates for 21/04/2026
</commit_message>
<xml_diff>
--- a/Suivi_Affaires_EGSA.xlsx
+++ b/Suivi_Affaires_EGSA.xlsx
@@ -1091,7 +1091,7 @@
       </c>
       <c r="G4" s="45" t="inlineStr">
         <is>
-          <t>RAPPEL demain après-midi 21/04 — Finaliser les lots CDC 2026 (AFF-004, 005, 006, 007 liées)</t>
+          <t>REPORT au 22/04 — Finaliser les lots CDC 2026 (AFF-004, 005, 006, 007 liées) — non traité le 21/04</t>
         </is>
       </c>
       <c r="H4" s="45" t="inlineStr">
@@ -1110,14 +1110,16 @@
         </is>
       </c>
       <c r="K4" s="52" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="L4" s="45" t="inlineStr">
         <is>
           <t>12/04 : Collègue a envoyé 10 lots par mail
 12/04 : Remarques faites sur les lots
 12/04 : Réunion tenue — questions en suspens identifiées par lot
-20/04/2026 — Planifié pour demain après-midi 21/04/2026. Les lots AFF-004/005/006/007 seront traités en même temps.</t>
+20/04/2026 — Planifié pour demain après-midi 21/04/2026. Les lots AFF-004/005/006/007 seront traités en même temps.
+21/04/2026 — Planifié pour cet après-midi 21/04. Finalisation des lots CDC 2026 avec AFF-004/005/006/007.
+21/04/2026 — Non traité (priorité donnée à AFF-011/009). Reporté au 22/04/2026.</t>
         </is>
       </c>
       <c r="M4" s="45" t="inlineStr">
@@ -1129,7 +1131,7 @@
       <c r="O4" s="46" t="n"/>
       <c r="P4" s="46" t="n"/>
       <c r="Q4" s="53" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="R4" s="46" t="inlineStr">
         <is>
@@ -1142,7 +1144,7 @@
         </is>
       </c>
       <c r="T4" s="53" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="U4" s="46" t="inlineStr">
         <is>
@@ -1191,7 +1193,7 @@
       </c>
       <c r="G5" s="47" t="inlineStr">
         <is>
-          <t>Traiter avec AFF-003 — demain après-midi 21/04/2026</t>
+          <t>REPORT au 22/04 — Traiter avec AFF-003 (Lot N°1 : PCs Bureau) — non traité le 21/04</t>
         </is>
       </c>
       <c r="H5" s="47" t="inlineStr">
@@ -1206,12 +1208,14 @@
       </c>
       <c r="J5" s="47" t="inlineStr"/>
       <c r="K5" s="50" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="L5" s="47" t="inlineStr">
         <is>
           <t>12/04 : Questions identifiées après réunion
-20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.</t>
+20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.
+21/04/2026 — Planifié pour cet après-midi 21/04 avec AFF-003.
+21/04/2026 — Non traité. Reporté au 22/04/2026 avec AFF-003.</t>
         </is>
       </c>
       <c r="M5" s="47" t="inlineStr">
@@ -1224,7 +1228,7 @@
       <c r="O5" s="47" t="n"/>
       <c r="P5" s="47" t="n"/>
       <c r="Q5" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="R5" s="47" t="inlineStr">
         <is>
@@ -1237,7 +1241,7 @@
         </is>
       </c>
       <c r="T5" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="U5" s="47" t="inlineStr">
         <is>
@@ -1286,7 +1290,7 @@
       </c>
       <c r="G6" s="47" t="inlineStr">
         <is>
-          <t>Traiter avec AFF-003 — demain après-midi 21/04/2026</t>
+          <t>REPORT au 22/04 — Traiter avec AFF-003 (Lot N°2 : PCs Architectes) — non traité le 21/04</t>
         </is>
       </c>
       <c r="H6" s="47" t="inlineStr">
@@ -1301,12 +1305,14 @@
       </c>
       <c r="J6" s="47" t="inlineStr"/>
       <c r="K6" s="50" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="L6" s="47" t="inlineStr">
         <is>
           <t>12/04 : Questions identifiées après réunion
-20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.</t>
+20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.
+21/04/2026 — Planifié pour cet après-midi 21/04 avec AFF-003.
+21/04/2026 — Non traité. Reporté au 22/04/2026 avec AFF-003.</t>
         </is>
       </c>
       <c r="M6" s="47" t="inlineStr">
@@ -1321,7 +1327,7 @@
       <c r="O6" s="47" t="n"/>
       <c r="P6" s="47" t="n"/>
       <c r="Q6" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="R6" s="47" t="inlineStr">
         <is>
@@ -1334,7 +1340,7 @@
         </is>
       </c>
       <c r="T6" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="U6" s="47" t="inlineStr">
         <is>
@@ -1383,7 +1389,7 @@
       </c>
       <c r="G7" s="47" t="inlineStr">
         <is>
-          <t>Traiter avec AFF-003 — demain après-midi 21/04/2026</t>
+          <t>REPORT au 22/04 — Traiter avec AFF-003 (Lot N°2 : Laptops Développeurs) — non traité le 21/04</t>
         </is>
       </c>
       <c r="H7" s="47" t="inlineStr">
@@ -1398,12 +1404,14 @@
       </c>
       <c r="J7" s="47" t="inlineStr"/>
       <c r="K7" s="50" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="L7" s="47" t="inlineStr">
         <is>
           <t>12/04 : Questions identifiées après réunion
-20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.</t>
+20/04/2026 — Sera traitée avec AFF-003 (CDC 2026) demain après-midi 21/04.
+21/04/2026 — Planifié pour cet après-midi 21/04 avec AFF-003.
+21/04/2026 — Non traité. Reporté au 22/04/2026 avec AFF-003.</t>
         </is>
       </c>
       <c r="M7" s="47" t="inlineStr">
@@ -1416,7 +1424,7 @@
       <c r="O7" s="47" t="n"/>
       <c r="P7" s="47" t="n"/>
       <c r="Q7" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="R7" s="47" t="inlineStr">
         <is>
@@ -1429,7 +1437,7 @@
         </is>
       </c>
       <c r="T7" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="U7" s="47" t="inlineStr">
         <is>
@@ -1674,7 +1682,7 @@
       </c>
       <c r="G10" s="47" t="inlineStr">
         <is>
-          <t>RAPPEL demain matin 21/04 — Analyser BD ERP avec collègues + préparer résumé commercial réunion 14/04</t>
+          <t>À CONTINUER demain 22/04 — Résumé module Commercial + analyse structure base de données (en cours depuis 21/04)</t>
         </is>
       </c>
       <c r="H10" s="47" t="inlineStr">
@@ -1689,7 +1697,7 @@
       </c>
       <c r="J10" s="47" t="n"/>
       <c r="K10" s="50" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="L10" s="47" t="inlineStr">
         <is>
@@ -1701,7 +1709,10 @@
 20/04/2026 — A COMMENCER : appeler collègue pour identifier BD production
 20/04/2026 — Base de données restaurée en local (.bak OK). BD identifiée : base des commerciaux en production. Prochaine étape : analyse structure + résumé commercial (en groupe avec collègues).
 20/04/2026 — Planifié pour demain matin 21/04/2026 : analyse BD structure + résumé commercial réunion commerciale du 14/04.
-20/04/2026 — Planifié pour demain matin 21/04/2026 : analyse structure BD + résumé commercial réunion du 14/04.</t>
+20/04/2026 — Planifié pour demain matin 21/04/2026 : analyse structure BD + résumé commercial réunion du 14/04.
+21/04/2026 — DÉMARRÉ ce matin, en parallèle avec AFF-011. Analyse structure BD + rédaction résumé commercial réunion 14/04.
+21/04/2026 — Travail commencé : analyse BD + résumé module Commercial. Non terminé en fin de journée. À continuer le 22/04/2026.
+21/04/2026 — Plan confirmé pour 22/04 : continuer résumé module Commercial + analyse structure BD. Travail en cours.</t>
         </is>
       </c>
       <c r="M10" s="47" t="inlineStr">
@@ -1713,7 +1724,7 @@
       <c r="O10" s="47" t="n"/>
       <c r="P10" s="47" t="n"/>
       <c r="Q10" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="R10" s="47" t="inlineStr">
         <is>
@@ -1726,7 +1737,7 @@
         </is>
       </c>
       <c r="T10" s="50" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="U10" s="47" t="n"/>
       <c r="V10" s="47" t="inlineStr">
@@ -1856,7 +1867,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Rédiger résumé métier commercial (réunion 15/04) + intégrer à la conception ERP — en coordination avec AFF-009</t>
+          <t>À CONTINUER demain 22/04 — Résumé module Commercial + analyse structure base de données (en cours depuis 21/04)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1871,13 +1882,16 @@
         <v>46127</v>
       </c>
       <c r="K12" s="51" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>15/04/2026 — Tâche ajoutée : entretien commercial à planifier aujourd'hui.
 20/04/2026 — Réunion avec commercial effectuée
-20/04/2026 — Réunion du 15/04 avec le commercial confirmée. Prochaine étape : rédiger résumé métier + l'intégrer à la conception ERP (lié AFF-009). Objectif : conception ERP complète et rigoureuse.</t>
+20/04/2026 — Réunion du 15/04 avec le commercial confirmée. Prochaine étape : rédiger résumé métier + l'intégrer à la conception ERP (lié AFF-009). Objectif : conception ERP complète et rigoureuse.
+21/04/2026 — DÉMARRÉ ce matin. Rédaction du résumé métier commercial + intégration conception ERP. En parallèle avec AFF-009. Peut se prolonger jusqu'au 22/04.
+21/04/2026 — Travail commencé : analyse BD + résumé module Commercial. Non terminé en fin de journée. À continuer le 22/04/2026.
+21/04/2026 — Plan confirmé pour 22/04 : continuer résumé module Commercial + analyse structure BD. Travail en cours.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1886,7 +1900,7 @@
         </is>
       </c>
       <c r="Q12" s="51" t="n">
-        <v>46127</v>
+        <v>46134</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1899,7 +1913,7 @@
         </is>
       </c>
       <c r="T12" s="51" t="n">
-        <v>46127</v>
+        <v>46134</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
@@ -2042,7 +2056,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>RAPPEL demain 21/04 — Relancer la directrice pour envoi des bilans mensuels J/F/M</t>
+          <t>RAPPEL demain 22/04 — Relancer la directrice pour envoi des bilans mensuels J/F/M — non traité le 21/04</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2054,17 +2068,19 @@
         <v>46132</v>
       </c>
       <c r="K14" s="51" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>20/04/2026 — CRÉÉ : Affaire de suivi pour les trois bilans mensuels
 Rappel quotidien jusqu'à complération
-20/04/2026 — Rappel programmé pour demain 21/04/2026.</t>
+20/04/2026 — Rappel programmé pour demain 21/04/2026.
+21/04/2026 — Rappel programmé pour cet après-midi 21/04/2026.
+21/04/2026 — Non traité. Rappel reporté au 22/04/2026.</t>
         </is>
       </c>
       <c r="Q14" s="51" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2077,7 +2093,7 @@
         </is>
       </c>
       <c r="T14" s="51" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>